<commit_message>
Auto update Vinculum data
</commit_message>
<xml_diff>
--- a/returns.xlsx
+++ b/returns.xlsx
@@ -4188,7 +4188,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Chemistry Med Easy | Notes, Formulas, Tips &amp; Tricks for NEET/JEE &amp; Board Exams | Pankaj Sir Chemistry Handwritten Notes</t>
+          <t xml:space="preserve">Chemistry Med Easy | Notes, Formulas, Tips &amp; Tricks for NEET/JEE &amp; Board Exams | Pankaj Sir Chemistry Handwritten Notes!</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -6636,7 +6636,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Chemistry Med Easy | Notes, Formulas, Tips &amp; Tricks for NEET/JEE &amp; Board Exams | Pankaj Sir Chemistry Handwritten Notes</t>
+          <t xml:space="preserve">Chemistry Med Easy | Notes, Formulas, Tips &amp; Tricks for NEET/JEE &amp; Board Exams | Pankaj Sir Chemistry Handwritten Notes!</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -22956,7 +22956,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Zoology Med Easy 2.0 For NEET and Board Exams 2025-26 | Flowcharts, Schematic Diagrams l Samapti Sinha Mahapatra Handwritten Notes</t>
+          <t xml:space="preserve">Zoology Med Easy 2.0 For NEET and Board Exams 2025-26 | Flowcharts, Schematic Diagrams l Samapti Sinha Mahapatra Handwritten Notes!</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -27852,7 +27852,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Absolute JEE Advanced Mathematics 2500+ Questions with Formula Sheet Latest Solved Paper and 3 Mock Tests | Covering All JEE Advanced Question Typology</t>
+          <t xml:space="preserve">Absolute JEE Advanced Mathematics 2500+ Questions with Formula Sheet Latest Solved Paper and 3 Mock Tests | Covering All JEE Advanced Question Typology--</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -31660,7 +31660,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Zoology Med Easy 2.0 For NEET and Board Exams 2025-26 | Flowcharts, Schematic Diagrams l Samapti Sinha Mahapatra Handwritten Notes</t>
+          <t xml:space="preserve">Zoology Med Easy 2.0 For NEET and Board Exams 2025-26 | Flowcharts, Schematic Diagrams l Samapti Sinha Mahapatra Handwritten Notes!</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -31932,7 +31932,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Chemistry Med Easy | Notes, Formulas, Tips &amp; Tricks for NEET/JEE &amp; Board Exams | Pankaj Sir Chemistry Handwritten Notes</t>
+          <t xml:space="preserve">Chemistry Med Easy | Notes, Formulas, Tips &amp; Tricks for NEET/JEE &amp; Board Exams | Pankaj Sir Chemistry Handwritten Notes!</t>
         </is>
       </c>
       <c t="inlineStr">

</xml_diff>